<commit_message>
BRD-covered green points re-classified black (BRD-00 and programme NFRs count)
Product owner decisions of 11-Oct-2026: green points that a BRD line asks for are BRD
requirements (black, in scope); offered OOTB, so no effort. BRD-11 OB-UA-01; BRD-06 G-19,
G-23; BRD-03 G-01, G-03, G-04, G-05; BRD-02 G-01. New BRD-covered tables in the annexes and
sheet 'BRD covered - OOTB' in the effort workbooks; CR register and RTM scope updated; BRD-11
e2e flow re-tagged. CR totals unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx
@@ -12,28 +12,31 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CR Effort" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beyond the BRD - OOTB" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration &amp; DM scope" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best practice (blue)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRD items to deliver" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRD covered - OOTB" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration &amp; DM scope" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best practice (blue)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRD items to deliver" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$4:$B$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary'!$A$4:$B$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Summary'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CR Effort'!$A$4:$Y$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'CR Effort'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Beyond the BRD - OOTB'!$A$4:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Beyond the BRD - OOTB'!$A$4:$G$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Beyond the BRD - OOTB'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Integration &amp; DM scope'!$A$4:$D$33</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Integration &amp; DM scope'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Best practice (blue)'!$A$4:$E$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Best practice (blue)'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'BRD items to deliver'!$A$4:$E$55</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'BRD items to deliver'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Lists'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'BRD covered - OOTB'!$A$4:$G$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'BRD covered - OOTB'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Integration &amp; DM scope'!$A$4:$D$33</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Integration &amp; DM scope'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Best practice (blue)'!$A$4:$E$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Best practice (blue)'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'BRD items to deliver'!$A$4:$E$55</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'BRD items to deliver'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Lists'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -364,7 +367,7 @@
     <from>
       <col>3</col>
       <colOff>0</colOff>
-      <row>29</row>
+      <row>30</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="971550" cy="285750"/>
@@ -677,7 +680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B4:E30"/>
+  <dimension ref="B4:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -843,7 +846,7 @@
         </is>
       </c>
       <c r="D21" s="14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22">
@@ -873,71 +876,86 @@
         </is>
       </c>
       <c r="D23" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>Integration &amp; DM scope</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>Covered by the Integration scope or the Data Migration scope (BRD-13): no CR cost here</t>
+          <t>BRD requirements (black in the FRS, in scope) that the iNXT BrokerVerse OOTB platform provides: no change request, no effort</t>
         </is>
       </c>
       <c r="D24" s="12" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>Integration &amp; DM scope</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Not in the BRD, the FRS or the OOTB platform: recommendations (Appendix W.6), not commitments</t>
+          <t>Covered by the Integration scope or the Data Migration scope (BRD-13): no CR cost here</t>
         </is>
       </c>
       <c r="D25" s="14" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>BRD items to deliver</t>
+          <t>Best practice (blue)</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>BRD requirements not fully met by the OOTB platform: in-scope delivery work for planning, not CRs</t>
+          <t>Not in the BRD, the FRS or the OOTB platform: recommendations (Appendix W.6), not commitments</t>
         </is>
       </c>
       <c r="D26" s="12" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="13" t="inlineStr">
         <is>
+          <t>BRD items to deliver</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>BRD requirements not fully met by the OOTB platform: in-scope delivery work for planning, not CRs</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="11" t="inlineStr">
+        <is>
           <t>Assumptions</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C28" s="12" t="inlineStr">
         <is>
           <t>Man-day, range and day rate used by the formulas</t>
         </is>
       </c>
-      <c r="D27" s="14" t="n">
+      <c r="D28" s="12" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="30" ht="26" customHeight="1">
-      <c r="B30" s="15" t="inlineStr">
+    <row r="31" ht="26" customHeight="1">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Prepared by iorta TechNXT for BDOI. Confidential – BDOI.</t>
         </is>
@@ -953,6 +971,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId9"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
@@ -965,11 +984,199 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Hours in a man-day</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>One man-day (md) = 8 working hours</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>Philippine peso</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>Estimate range (plus or minus)</t>
+        </is>
+      </c>
+      <c r="B6" s="26" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>Each total is an estimate within plus or minus 20%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>DayRate (PHP per man-day)</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="n"/>
+      <c r="C7" s="25" t="inlineStr">
+        <is>
+          <t>Enter the agreed day rate; the cost columns follow by formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>OOTB baseline</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>brokerverse-platform</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>iNXT BrokerVerse OOTB platform (brokerverse-platform), with the programme Feature List (column OOTB platform) as a cross-check</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Platform size</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>Effort from the size of the platform parts each change touches and a similar existing function; for a Partial feature, the missing part only</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Not change requests</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>BRD requirements (in scope), Integration scope and Data Migration scope items, best-practice recommendations</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Excluded</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>BDOI decisions and inputs, BDOI testing time, infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>Validity</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>30 days</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Estimated again if the scope of a change request changes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1083,7 +1290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1755,17 +1962,17 @@
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Integration &amp; DM scope</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>No.</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>Interface or data load</t>
+          <t>Former green point</t>
         </is>
       </c>
       <c r="D39" s="12" t="inlineStr"/>
@@ -1773,39 +1980,35 @@
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>Integration &amp; DM scope</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Scope</t>
+          <t>Point</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>Integration or Data Migration</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="inlineStr">
-        <is>
-          <t>Integration scope, Data Migration scope</t>
-        </is>
-      </c>
+          <t>The point of the FRS</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>Integration &amp; DM scope</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>What</t>
+          <t>FRS reference</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>What is exchanged or loaded</t>
+          <t>FR item or annex</t>
         </is>
       </c>
       <c r="D41" s="12" t="inlineStr"/>
@@ -1813,17 +2016,17 @@
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Integration &amp; DM scope</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Where in the FRS</t>
+          <t>BRD line</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>Annex</t>
+          <t>The BRD line that asks for it (BRD, BRD-00 or programme-wide NFR)</t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr"/>
@@ -1831,17 +2034,17 @@
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Feature List ID / OOTB status</t>
         </is>
       </c>
       <c r="C43" s="12" t="inlineStr">
         <is>
-          <t>Best practice</t>
+          <t>Programme Feature List, column OOTB platform</t>
         </is>
       </c>
       <c r="D43" s="12" t="inlineStr"/>
@@ -1849,17 +2052,17 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>Practice</t>
+          <t>OOTB evidence</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>Insurance-broking practice</t>
+          <t>Screen or function of brokerverse-platform</t>
         </is>
       </c>
       <c r="D44" s="14" t="inlineStr"/>
@@ -1867,17 +2070,17 @@
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>BRD covered - OOTB</t>
         </is>
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>Why it matters for a broker</t>
+          <t>Effort (md)</t>
         </is>
       </c>
       <c r="C45" s="12" t="inlineStr">
         <is>
-          <t>Philippine market where relevant</t>
+          <t>Zero: offered OOTB</t>
         </is>
       </c>
       <c r="D45" s="12" t="inlineStr"/>
@@ -1885,57 +2088,57 @@
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>Integration &amp; DM scope</t>
         </is>
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>Suggested priority</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>High / Medium / Low</t>
-        </is>
-      </c>
-      <c r="D46" s="14" t="inlineStr">
-        <is>
-          <t>High, Medium, Low</t>
-        </is>
-      </c>
+          <t>Interface or data load</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>Best practice (blue)</t>
+          <t>Integration &amp; DM scope</t>
         </is>
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>Indicative man-days</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>Indicative; not in the CR total</t>
-        </is>
-      </c>
-      <c r="D47" s="12" t="inlineStr"/>
+          <t>Integration or Data Migration</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>Integration scope, Data Migration scope</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>BRD items to deliver</t>
+          <t>Integration &amp; DM scope</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>BRD ID</t>
+          <t>What</t>
         </is>
       </c>
       <c r="C48" s="14" t="inlineStr">
         <is>
-          <t>BRD requirement</t>
+          <t>What is exchanged or loaded</t>
         </is>
       </c>
       <c r="D48" s="14" t="inlineStr"/>
@@ -1943,17 +2146,17 @@
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>BRD items to deliver</t>
+          <t>Integration &amp; DM scope</t>
         </is>
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>BRD requirement</t>
+          <t>Where in the FRS</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>Text of the BRD</t>
+          <t>Annex</t>
         </is>
       </c>
       <c r="D49" s="12" t="inlineStr"/>
@@ -1961,17 +2164,17 @@
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>BRD items to deliver</t>
+          <t>Best practice (blue)</t>
         </is>
       </c>
       <c r="B50" s="18" t="inlineStr">
         <is>
-          <t>Fit</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>Fit class of the fit-gap workbook</t>
+          <t>Best practice</t>
         </is>
       </c>
       <c r="D50" s="14" t="inlineStr"/>
@@ -1979,17 +2182,17 @@
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>BRD items to deliver</t>
+          <t>Best practice (blue)</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>What iNXT BrokerVerse offers out of the box</t>
+          <t>Practice</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>OOTB capability</t>
+          <t>Insurance-broking practice</t>
         </is>
       </c>
       <c r="D51" s="12" t="inlineStr"/>
@@ -1997,23 +2200,153 @@
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
+          <t>Best practice (blue)</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>Why it matters for a broker</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>Philippine market where relevant</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Best practice (blue)</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>Suggested priority</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>High / Medium / Low</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>High, Medium, Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Best practice (blue)</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>Indicative man-days</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Indicative; not in the CR total</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="12" t="inlineStr">
+        <is>
           <t>BRD items to deliver</t>
         </is>
       </c>
-      <c r="B52" s="18" t="inlineStr">
+      <c r="B55" s="17" t="inlineStr">
+        <is>
+          <t>BRD ID</t>
+        </is>
+      </c>
+      <c r="C55" s="12" t="inlineStr">
+        <is>
+          <t>BRD requirement</t>
+        </is>
+      </c>
+      <c r="D55" s="12" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>BRD items to deliver</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>BRD requirement</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Text of the BRD</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="12" t="inlineStr">
+        <is>
+          <t>BRD items to deliver</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="inlineStr">
+        <is>
+          <t>Fit</t>
+        </is>
+      </c>
+      <c r="C57" s="12" t="inlineStr">
+        <is>
+          <t>Fit class of the fit-gap workbook</t>
+        </is>
+      </c>
+      <c r="D57" s="12" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>BRD items to deliver</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>What iNXT BrokerVerse offers out of the box</t>
+        </is>
+      </c>
+      <c r="C58" s="14" t="inlineStr">
+        <is>
+          <t>OOTB capability</t>
+        </is>
+      </c>
+      <c r="D58" s="14" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="inlineStr">
+        <is>
+          <t>BRD items to deliver</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
         <is>
           <t>Planning man-days</t>
         </is>
       </c>
-      <c r="C52" s="14" t="inlineStr">
+      <c r="C59" s="12" t="inlineStr">
         <is>
           <t>For the points of BDOI's FRS covered by a BRD line</t>
         </is>
       </c>
-      <c r="D52" s="14" t="inlineStr"/>
+      <c r="D59" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D52"/>
+  <autoFilter ref="A4:D59"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -2034,7 +2367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -2078,154 +2411,164 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>Change requests (orange)</t>
+          <t>BRD requirements offered OOTB (black, in scope, no effort)</t>
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
+          <t>Change requests (orange)</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
           <t>Man-days: Analysis &amp; design</t>
         </is>
       </c>
-      <c r="B7" s="12">
+      <c r="B8" s="12">
         <f>SUM('CR Effort'!M5:M6)</f>
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>Man-days: Backend</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B9" s="12">
         <f>SUM('CR Effort'!N5:N6)</f>
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Man-days: Frontend</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B10" s="12">
         <f>SUM('CR Effort'!O5:O6)</f>
         <v/>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Man-days: Testing</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B11" s="12">
         <f>SUM('CR Effort'!P5:P6)</f>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Man-days: Documentation / UAT support</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B12" s="12">
         <f>SUM('CR Effort'!Q5:Q6)</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Total change request man-days</t>
         </is>
       </c>
-      <c r="B12" s="12">
+      <c r="B13" s="12">
         <f>SUM('CR Effort'!R5:R6)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Range low (-20%)</t>
         </is>
       </c>
-      <c r="B13" s="12">
+      <c r="B14" s="12">
         <f>SUM('CR Effort'!S5:S6)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Range high (+20%)</t>
         </is>
       </c>
-      <c r="B14" s="12">
+      <c r="B15" s="12">
         <f>SUM('CR Effort'!T5:T6)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Cost in PHP at the day rate of the Assumptions sheet</t>
         </is>
       </c>
-      <c r="B15" s="12">
+      <c r="B16" s="12">
         <f>SUM('CR Effort'!U5:U6)</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Items covered by the Integration or Data Migration scope (no CR cost)</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>29</v>
-      </c>
-    </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Best-practice recommendations (blue; indicative, not in the CR total)</t>
+          <t>Items covered by the Integration or Data Migration scope (no CR cost)</t>
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>3</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
+          <t>Best-practice recommendations (blue; indicative, not in the CR total)</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
           <t>Best-practice indicative man-days (not in the CR total)</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B19" s="12" t="n">
         <v>15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B18"/>
+  <autoFilter ref="A4:B19"/>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:B518">
+  <conditionalFormatting sqref="A5:B519">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
@@ -2777,7 +3120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2852,17 +3195,17 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>G-01</t>
+          <t>G-01b</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Scheduled daily run of the Daily Cash Reconciliation Reports</t>
+          <t>Scheduled weekly run of the Unapplied Premium Payment Transaction report</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>FRS.CSH.09.02.10; Appendix M</t>
+          <t>FRS.CSH.09.02.11; Appendix M</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -2884,47 +3227,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>G-01b</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Scheduled weekly run of the Unapplied Premium Payment Transaction report</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>FRS.CSH.09.02.11; Appendix M</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>RPT-007 Available (user-scheduled reports with recipients)</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Reports &gt; Schedules: timing, format and recipients</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Not in BRD</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:G6"/>
+  <autoFilter ref="A4:G5"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G506">
+  <conditionalFormatting sqref="A5:G505">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
@@ -2944,6 +3252,143 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>BRD covered - OOTB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>BRD requirements (black in the FRS, in scope) that the iNXT BrokerVerse OOTB platform provides: no change request, no effort</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1">
+      <c r="A3" s="20" t="n"/>
+      <c r="B3" s="20" t="n"/>
+      <c r="C3" s="20" t="n"/>
+      <c r="D3" s="20" t="n"/>
+      <c r="E3" s="20" t="n"/>
+      <c r="F3" s="20" t="n"/>
+      <c r="G3" s="20" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Point</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>FRS reference</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>BRD line</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Feature List ID / OOTB status</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>OOTB evidence</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>Effort (md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>G-01</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Scheduled daily run of the Daily Cash Reconciliation Reports</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>FRS.CSH.09.02.10; Appendix M</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>CSHID.023 "Capability to generate reports. See Cashiering Reports list under Annex"; Report List (Operations - Cashiering): "Daily Cash Reconciliation Reports - Summarizes daily cash receipts and deposits", frequency "Daily"</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>RPT-007 Available (user-scheduled reports with recipients)</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Reports &gt; Schedules: timing, format and recipients</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G5"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A5:G505">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Effort Estimate&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3667,7 +4112,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3835,7 +4280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5098,192 +5543,4 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>Assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="24" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="25" t="inlineStr">
-        <is>
-          <t>Hours in a man-day</t>
-        </is>
-      </c>
-      <c r="B4" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>One man-day (md) = 8 working hours</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="25" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B5" s="25" t="inlineStr">
-        <is>
-          <t>PHP</t>
-        </is>
-      </c>
-      <c r="C5" s="25" t="inlineStr">
-        <is>
-          <t>Philippine peso</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="25" t="inlineStr">
-        <is>
-          <t>Estimate range (plus or minus)</t>
-        </is>
-      </c>
-      <c r="B6" s="26" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>Each total is an estimate within plus or minus 20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t>DayRate (PHP per man-day)</t>
-        </is>
-      </c>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>Enter the agreed day rate; the cost columns follow by formula</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>OOTB baseline</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>brokerverse-platform</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
-        <is>
-          <t>iNXT BrokerVerse OOTB platform (brokerverse-platform), with the programme Feature List (column OOTB platform) as a cross-check</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>Basis</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="inlineStr">
-        <is>
-          <t>Platform size</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>Effort from the size of the platform parts each change touches and a similar existing function; for a Partial feature, the missing part only</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>Not change requests</t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>BRD requirements (in scope), Integration scope and Data Migration scope items, best-practice recommendations</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>Excluded</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>BDOI decisions and inputs, BDOI testing time, infrastructure</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="25" t="inlineStr">
-        <is>
-          <t>Validity</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="inlineStr">
-        <is>
-          <t>30 days</t>
-        </is>
-      </c>
-      <c r="C12" s="25" t="inlineStr">
-        <is>
-          <t>Estimated again if the scope of a change request changes</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>